<commit_message>
MJ: add POL campaigns tab (conversions) to ad-data workbook
</commit_message>
<xml_diff>
--- a/outputs/monkey-joes/MJ-Ad-Data-AllTime.xlsx
+++ b/outputs/monkey-joes/MJ-Ad-Data-AllTime.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Google WP - Billing" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Google - Monthly Spend" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Google WP - Campaigns" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Facebook &amp; Instagram" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Google POL - Daily Impr" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Google POL - Campaigns" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Facebook &amp; Instagram" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Google POL - Daily Impr" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,9 +25,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00;(&quot;$&quot;#,##0.00)"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -130,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,7 +144,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,16 +155,21 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -630,7 +636,6 @@
         <v>2056.58</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -677,7 +682,7 @@
       <c r="C12" s="9" t="n">
         <v>3376</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="31" t="n">
         <v>54</v>
       </c>
       <c r="E12" s="11" t="n">
@@ -696,7 +701,7 @@
       <c r="C13" s="9" t="n">
         <v>1406</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="31" t="n">
         <v>51</v>
       </c>
       <c r="E13" s="11" t="n">
@@ -710,7 +715,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -760,7 +764,6 @@
         <v>3.59</v>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -916,7 +919,7 @@
         <v>1.23</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G3" s="16" t="n">
         <v>344.81</v>
@@ -1009,7 +1012,7 @@
         <v>8.779999999999999</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G6" s="16" t="n">
         <v>328.24</v>
@@ -1102,7 +1105,7 @@
         <v>8.949999999999999</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G9" s="16" t="n">
         <v>305.47</v>
@@ -1164,7 +1167,7 @@
         <v>6.52</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G11" s="16" t="n">
         <v>282.14</v>
@@ -1195,7 +1198,7 @@
         <v>14.49</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G12" s="16" t="n">
         <v>275.62</v>
@@ -1257,7 +1260,7 @@
         <v>4.25</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G14" s="16" t="n">
         <v>248.45</v>
@@ -1319,7 +1322,7 @@
         <v>9.06</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G16" s="16" t="n">
         <v>243.43</v>
@@ -1598,7 +1601,7 @@
         <v>3.26</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G25" s="16" t="n">
         <v>165.1</v>
@@ -1629,7 +1632,7 @@
         <v>11.24</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G26" s="16" t="n">
         <v>161.84</v>
@@ -1815,7 +1818,7 @@
         <v>12.56</v>
       </c>
       <c r="F32" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G32" s="16" t="n">
         <v>108.74</v>
@@ -1908,7 +1911,7 @@
         <v>3.64</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G35" s="16" t="n">
         <v>78.54000000000001</v>
@@ -2185,7 +2188,7 @@
         <v>6.1</v>
       </c>
       <c r="F44" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G44" s="16" t="n">
         <v>347.55</v>
@@ -2772,7 +2775,7 @@
         <v>5.86</v>
       </c>
       <c r="F63" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G63" s="16" t="n">
         <v>377.12</v>
@@ -2803,7 +2806,7 @@
         <v>7.19</v>
       </c>
       <c r="F64" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G64" s="16" t="n">
         <v>371.26</v>
@@ -2927,7 +2930,7 @@
         <v>10.94</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G68" s="16" t="n">
         <v>341.45</v>
@@ -2989,7 +2992,7 @@
         <v>9.539999999999999</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G70" s="16" t="n">
         <v>324.41</v>
@@ -3020,7 +3023,7 @@
         <v>7.95</v>
       </c>
       <c r="F71" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G71" s="16" t="n">
         <v>314.87</v>
@@ -3144,7 +3147,7 @@
         <v>10.93</v>
       </c>
       <c r="F75" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G75" s="16" t="n">
         <v>275.48</v>
@@ -3578,7 +3581,7 @@
         <v>19.99</v>
       </c>
       <c r="F89" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G89" s="16" t="n">
         <v>63.68</v>
@@ -3671,7 +3674,7 @@
         <v>9.81</v>
       </c>
       <c r="F92" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G92" s="16" t="n">
         <v>9.81</v>
@@ -3944,7 +3947,7 @@
         <v>1.68</v>
       </c>
       <c r="F101" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G101" s="16" t="n">
         <v>314.74</v>
@@ -4037,7 +4040,7 @@
         <v>3.44</v>
       </c>
       <c r="F104" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G104" s="16" t="n">
         <v>302.54</v>
@@ -4192,7 +4195,7 @@
         <v>20.57</v>
       </c>
       <c r="F109" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G109" s="16" t="n">
         <v>219.5</v>
@@ -4223,7 +4226,7 @@
         <v>33.34</v>
       </c>
       <c r="F110" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G110" s="16" t="n">
         <v>198.93</v>
@@ -4254,7 +4257,7 @@
         <v>7.13</v>
       </c>
       <c r="F111" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G111" s="16" t="n">
         <v>165.59</v>
@@ -4440,7 +4443,7 @@
         <v>8.529999999999999</v>
       </c>
       <c r="F117" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G117" s="16" t="n">
         <v>86.77</v>
@@ -4471,7 +4474,7 @@
         <v>19.36</v>
       </c>
       <c r="F118" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G118" s="16" t="n">
         <v>78.23999999999999</v>
@@ -4655,7 +4658,7 @@
         <v>4.32</v>
       </c>
       <c r="F124" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G124" s="16" t="n">
         <v>159.41</v>
@@ -4779,7 +4782,7 @@
         <v>9.99</v>
       </c>
       <c r="F128" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G128" s="16" t="n">
         <v>65.12</v>
@@ -4841,7 +4844,7 @@
         <v>14.39</v>
       </c>
       <c r="F130" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G130" s="16" t="n">
         <v>48.64</v>
@@ -4903,7 +4906,7 @@
         <v>12.96</v>
       </c>
       <c r="F132" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G132" s="16" t="n">
         <v>31.92</v>
@@ -5455,7 +5458,7 @@
         <v>7.89</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G13" s="16" t="n">
         <v>274.65</v>
@@ -5765,7 +5768,7 @@
         <v>12.34</v>
       </c>
       <c r="F23" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G23" s="16" t="n">
         <v>194.61</v>
@@ -5920,7 +5923,7 @@
         <v>2.98</v>
       </c>
       <c r="F28" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G28" s="16" t="n">
         <v>131.74</v>
@@ -6106,7 +6109,7 @@
         <v>8.24</v>
       </c>
       <c r="F34" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G34" s="16" t="n">
         <v>93.36</v>
@@ -6137,7 +6140,7 @@
         <v>10.07</v>
       </c>
       <c r="F35" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G35" s="16" t="n">
         <v>85.12</v>
@@ -6323,7 +6326,7 @@
         <v>8.18</v>
       </c>
       <c r="F41" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G41" s="16" t="n">
         <v>28.36</v>
@@ -6782,7 +6785,7 @@
         <v>7.77</v>
       </c>
       <c r="F56" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G56" s="16" t="n">
         <v>94.68000000000001</v>
@@ -6875,7 +6878,7 @@
         <v>5.8</v>
       </c>
       <c r="F59" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G59" s="16" t="n">
         <v>71.48</v>
@@ -6968,7 +6971,7 @@
         <v>7.05</v>
       </c>
       <c r="F62" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G62" s="16" t="n">
         <v>37.59</v>
@@ -7121,7 +7124,7 @@
         <v>9.93</v>
       </c>
       <c r="F67" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G67" s="16" t="n">
         <v>361.93</v>
@@ -7183,7 +7186,7 @@
         <v>15.07</v>
       </c>
       <c r="F69" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G69" s="16" t="n">
         <v>347.04</v>
@@ -7214,7 +7217,7 @@
         <v>9.24</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G70" s="16" t="n">
         <v>331.97</v>
@@ -7245,7 +7248,7 @@
         <v>9.32</v>
       </c>
       <c r="F71" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G71" s="16" t="n">
         <v>322.73</v>
@@ -7276,7 +7279,7 @@
         <v>6.7</v>
       </c>
       <c r="F72" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G72" s="16" t="n">
         <v>313.41</v>
@@ -7338,7 +7341,7 @@
         <v>4.75</v>
       </c>
       <c r="F74" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G74" s="16" t="n">
         <v>298.87</v>
@@ -7431,7 +7434,7 @@
         <v>6.82</v>
       </c>
       <c r="F77" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G77" s="16" t="n">
         <v>274.28</v>
@@ -8175,7 +8178,7 @@
         <v>9.58</v>
       </c>
       <c r="F101" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G101" s="16" t="n">
         <v>73.48999999999999</v>
@@ -8607,7 +8610,7 @@
         <v>13.5</v>
       </c>
       <c r="F115" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G115" s="16" t="n">
         <v>128.8</v>
@@ -8731,7 +8734,7 @@
         <v>10.46</v>
       </c>
       <c r="F119" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G119" s="16" t="n">
         <v>72.25</v>
@@ -9008,7 +9011,7 @@
         <v>17.59</v>
       </c>
       <c r="F128" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G128" s="16" t="n">
         <v>136.77</v>
@@ -9194,7 +9197,7 @@
         <v>16.42</v>
       </c>
       <c r="F134" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G134" s="16" t="n">
         <v>19.52</v>
@@ -9376,7 +9379,7 @@
         <v>29.95</v>
       </c>
       <c r="F140" s="16" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G140" s="16" t="n">
         <v>89.15000000000001</v>
@@ -9788,7 +9791,7 @@
           <t>MJ — BOGO — Winter Park</t>
         </is>
       </c>
-      <c r="B2" s="21" t="n">
+      <c r="B2" s="32" t="n">
         <v>7</v>
       </c>
       <c r="C2" s="22" t="n">
@@ -9806,7 +9809,7 @@
       <c r="G2" s="24" t="n">
         <v>554.76</v>
       </c>
-      <c r="H2" s="25" t="n">
+      <c r="H2" s="33" t="n">
         <v>12.83</v>
       </c>
       <c r="I2" s="24" t="n">
@@ -9824,7 +9827,7 @@
           <t>MJ — 50% Off — Winter Park</t>
         </is>
       </c>
-      <c r="B3" s="21" t="n">
+      <c r="B3" s="32" t="n">
         <v>10</v>
       </c>
       <c r="C3" s="22" t="n">
@@ -9842,7 +9845,7 @@
       <c r="G3" s="24" t="n">
         <v>877.1799999999999</v>
       </c>
-      <c r="H3" s="25" t="n">
+      <c r="H3" s="33" t="n">
         <v>41.17</v>
       </c>
       <c r="I3" s="24" t="n">
@@ -9860,7 +9863,7 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B4" s="26" t="n"/>
+      <c r="B4" s="34" t="n"/>
       <c r="C4" s="27" t="n">
         <v>60713</v>
       </c>
@@ -9876,7 +9879,7 @@
       <c r="G4" s="29" t="n">
         <v>1431.94</v>
       </c>
-      <c r="H4" s="30" t="n">
+      <c r="H4" s="35" t="n">
         <v>54</v>
       </c>
       <c r="I4" s="29" t="n">
@@ -9890,6 +9893,193 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Daily budget</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>CTR</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Avg CPC</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Conversions</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Cost / conv.</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Bid strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>MJ — BOGO — Pointe Orlando</t>
+        </is>
+      </c>
+      <c r="B2" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" s="22" t="n">
+        <v>11872</v>
+      </c>
+      <c r="D2" s="22" t="n">
+        <v>615</v>
+      </c>
+      <c r="E2" s="23" t="n">
+        <v>0.05180256064690027</v>
+      </c>
+      <c r="F2" s="24" t="n">
+        <v>1.23660162601626</v>
+      </c>
+      <c r="G2" s="24" t="n">
+        <v>760.51</v>
+      </c>
+      <c r="H2" s="33" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="I2" s="24" t="n">
+        <v>37.40826364977865</v>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>Maximize Conversions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>MJ — 50% Off — Pointe Orlando</t>
+        </is>
+      </c>
+      <c r="B3" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" s="22" t="n">
+        <v>14144</v>
+      </c>
+      <c r="D3" s="22" t="n">
+        <v>791</v>
+      </c>
+      <c r="E3" s="23" t="n">
+        <v>0.05592477375565611</v>
+      </c>
+      <c r="F3" s="24" t="n">
+        <v>1.102085967130215</v>
+      </c>
+      <c r="G3" s="24" t="n">
+        <v>871.75</v>
+      </c>
+      <c r="H3" s="33" t="n">
+        <v>30.67</v>
+      </c>
+      <c r="I3" s="24" t="n">
+        <v>28.42354091946527</v>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>Maximize Conversions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B4" s="34" t="n"/>
+      <c r="C4" s="27" t="n">
+        <v>26016</v>
+      </c>
+      <c r="D4" s="27" t="n">
+        <v>1406</v>
+      </c>
+      <c r="E4" s="28" t="n">
+        <v>0.05404366543665436</v>
+      </c>
+      <c r="F4" s="29" t="n">
+        <v>1.160924608819346</v>
+      </c>
+      <c r="G4" s="29" t="n">
+        <v>1632.26</v>
+      </c>
+      <c r="H4" s="35" t="n">
+        <v>51</v>
+      </c>
+      <c r="I4" s="29" t="n">
+        <v>32.00509803921569</v>
+      </c>
+      <c r="J4" s="19" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>POL campaign performance as of ~Jul 13 (billing/spend elsewhere is current to Jul 21).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10098,7 +10288,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>